<commit_message>
Also had to remove the link from the test file, for same reasons as previous commit
</commit_message>
<xml_diff>
--- a/test/fixtures/Test_format_good_Seq.xlsx
+++ b/test/fixtures/Test_format_good_Seq.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jc2017/Documents/MyRepos/safedata_validator/test/fixtures/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jc2017/Repositories/safedata_validator/test/fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C19AD6E-3EAD-F841-AB85-AC00A78FBE3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECDDD9A6-A806-C947-AD26-EDB27E1EFE18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="1060" windowWidth="27860" windowHeight="15840" xr2:uid="{819B57D8-7F20-471A-9405-EB60A28E68AA}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8319" uniqueCount="1458">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8318" uniqueCount="1457">
   <si>
     <t>Kingdom</t>
   </si>
@@ -4404,9 +4404,6 @@
   </si>
   <si>
     <t>ASV_132</t>
-  </si>
-  <si>
-    <t>https://www.arb-silva.de</t>
   </si>
 </sst>
 </file>
@@ -5108,9 +5105,6 @@
         <v>1439</v>
       </c>
       <c r="B31" s="5"/>
-      <c r="C31" t="s">
-        <v>1457</v>
-      </c>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>